<commit_message>
Updated files and script added
</commit_message>
<xml_diff>
--- a/Screens/Empresas.xlsx
+++ b/Screens/Empresas.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://academiafaedupt-my.sharepoint.com/personal/sbclemente_academiafa_edu_pt/Documents/Gigs/Financials/Meu/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://academiafaedupt-my.sharepoint.com/personal/sbclemente_academiafa_edu_pt/Documents/Gigs/WorkingFolder/Finance_Shared/Screens/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="117" documentId="8_{9D4384EC-C571-48BD-9208-0F280D17D66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{084167A0-BC2B-4ECA-9E9E-F2F726C81AEB}"/>
+  <xr:revisionPtr revIDLastSave="145" documentId="8_{9D4384EC-C571-48BD-9208-0F280D17D66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18633644-B1DB-47D4-9C40-F2B10BC097F2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{53EA3CC3-8788-4E7A-9C67-93E784C0731C}"/>
+    <workbookView xWindow="3375" yWindow="0" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{53EA3CC3-8788-4E7A-9C67-93E784C0731C}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
     <sheet name="Bancos" sheetId="3" r:id="rId2"/>
     <sheet name="Construtoras" sheetId="2" r:id="rId3"/>
+    <sheet name="Jornadas Civil" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -56,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
   <si>
     <t>Santos Barosa</t>
   </si>
@@ -149,13 +150,37 @@
   </si>
   <si>
     <t>Barclays</t>
+  </si>
+  <si>
+    <t>Empresa</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Placer</t>
+  </si>
+  <si>
+    <t>Socials</t>
+  </si>
+  <si>
+    <t>https://www.placer.pt/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenBook </t>
+  </si>
+  <si>
+    <t>https://openbook.pt/</t>
+  </si>
+  <si>
+    <t>Huild</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,6 +191,20 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -187,15 +226,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperligação" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1014,21 +1058,29 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC92488-F630-4736-BA9E-1D241702CD1F}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="B2:C5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="2" spans="2:3" s="3" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C5" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1039,28 +1091,94 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCBAD2D8-BC6B-4279-A551-520ED56A8CDE}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="B2:C11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="2" spans="2:3" s="3" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B9" s="2"/>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C933A3F-80EF-46EA-8E7C-75BF8DC8BA16}">
+  <dimension ref="B25:D28"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="9.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B26" s="4">
+        <v>46083</v>
+      </c>
+      <c r="C26" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B27" s="4">
+        <v>46083</v>
+      </c>
+      <c r="C27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B28" s="4">
+        <v>46083</v>
+      </c>
+      <c r="C28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D26" r:id="rId1" xr:uid="{4513792D-0E83-4043-B3E1-58ADFD1B9EB2}"/>
+    <hyperlink ref="D27" r:id="rId2" xr:uid="{F88F6C33-846E-4BE6-9610-26860C597949}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>